<commit_message>
#9 BOM eSpark and JLCPCB BOM Completed
</commit_message>
<xml_diff>
--- a/BOM/JLCPCB-BOM.xlsx
+++ b/BOM/JLCPCB-BOM.xlsx
@@ -132,7 +132,7 @@
     <t>270K</t>
   </si>
   <si>
-    <t>B3U-1000P</t>
+    <t>TS-1109S-C-B</t>
   </si>
   <si>
     <t>DSIC01LSGET</t>
@@ -420,12 +420,18 @@
     <t>C106256</t>
   </si>
   <si>
+    <t>C2936601</t>
+  </si>
+  <si>
     <t>C338080</t>
   </si>
   <si>
     <t>C277476</t>
   </si>
   <si>
+    <t>C441758</t>
+  </si>
+  <si>
     <t>C326057</t>
   </si>
   <si>
@@ -480,9 +486,6 @@
     <t>C105428</t>
   </si>
   <si>
-    <t>C137211</t>
-  </si>
-  <si>
     <t>C107701</t>
   </si>
   <si>
@@ -504,7 +507,7 @@
     <t>C724006</t>
   </si>
   <si>
-    <t>C231329</t>
+    <t>C381037</t>
   </si>
   <si>
     <t>C54948</t>
@@ -543,19 +546,16 @@
     <t>C129522</t>
   </si>
   <si>
+    <t>C506795</t>
+  </si>
+  <si>
+    <t>C95177</t>
+  </si>
+  <si>
     <t>C15651</t>
   </si>
   <si>
-    <t>C95177</t>
-  </si>
-  <si>
-    <t>C506795</t>
-  </si>
-  <si>
-    <t>C92487</t>
-  </si>
-  <si>
-    <t>C881842</t>
+    <t>C431873</t>
   </si>
 </sst>
 </file>
@@ -1105,7 +1105,7 @@
         <v>104</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>177</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1119,7 +1119,7 @@
         <v>107</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1133,7 +1133,7 @@
         <v>104</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1147,7 +1147,7 @@
         <v>106</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>178</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1161,7 +1161,7 @@
         <v>104</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1174,8 +1174,8 @@
       <c r="C12" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>136</v>
+      <c r="D12" s="4" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1188,8 +1188,8 @@
       <c r="C13" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>137</v>
+      <c r="D13" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1202,8 +1202,8 @@
       <c r="C14" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>138</v>
+      <c r="D14" s="4" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1217,7 +1217,7 @@
         <v>108</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1231,7 +1231,7 @@
         <v>109</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1245,7 +1245,7 @@
         <v>110</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>111</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1273,7 +1273,7 @@
         <v>111</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1287,7 +1287,7 @@
         <v>18</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1301,7 +1301,7 @@
         <v>19</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1315,7 +1315,7 @@
         <v>20</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1329,7 +1329,7 @@
         <v>21</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1343,7 +1343,7 @@
         <v>112</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1357,7 +1357,7 @@
         <v>113</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1371,7 +1371,7 @@
         <v>113</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1385,7 +1385,7 @@
         <v>114</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1399,7 +1399,7 @@
         <v>114</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1413,7 +1413,7 @@
         <v>114</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1427,7 +1427,7 @@
         <v>114</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1441,7 +1441,7 @@
         <v>115</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>153</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1455,7 +1455,7 @@
         <v>114</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1469,7 +1469,7 @@
         <v>114</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1483,7 +1483,7 @@
         <v>114</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1497,7 +1497,7 @@
         <v>114</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1511,7 +1511,7 @@
         <v>114</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1525,7 +1525,7 @@
         <v>114</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1539,7 +1539,7 @@
         <v>114</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1553,7 +1553,7 @@
         <v>37</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1567,7 +1567,7 @@
         <v>38</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1581,7 +1581,7 @@
         <v>39</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1595,7 +1595,7 @@
         <v>116</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1609,7 +1609,7 @@
         <v>117</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1623,7 +1623,7 @@
         <v>118</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1637,7 +1637,7 @@
         <v>119</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1651,7 +1651,7 @@
         <v>120</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1665,7 +1665,7 @@
         <v>121</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1679,7 +1679,7 @@
         <v>122</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1693,7 +1693,7 @@
         <v>123</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1707,7 +1707,7 @@
         <v>124</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1721,7 +1721,7 @@
         <v>125</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1735,7 +1735,7 @@
         <v>126</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>